<commit_message>
El lector de la CLI de Supabase entiende las filas sueltas y las envueltas
Al regenerar los informes desde la terminal, la CLI devolvió las filas como un
array a secas y el lector solo entendía el objeto con «rows» y el aviso de
datos no fiables, que es lo que devuelve desde el resto de sitios. Se localiza
el JSON por su primer corchete o llave, se cierra en el último y valen las dos
formas; las líneas sueltas de la CLI alrededor no molestan.
</commit_message>
<xml_diff>
--- a/docs/dominio-metrico/migracion/cuestionarios/el-caballero-de-olmedo.xlsx
+++ b/docs/dominio-metrico/migracion/cuestionarios/el-caballero-de-olmedo.xlsx
@@ -21,25 +21,25 @@
     <t>Migración métrica · El caballero de Olmedo</t>
   </si>
   <si>
-    <t>Para María Isabel Cuena · generado el 2026-09-19</t>
-  </si>
-  <si>
-    <t>El Excel tiene cinco pestañas. En tres de ellas hay que escribir —Responder, Confirmar y Desviaciones— y las otras dos son de consulta: Secuencias, con todo lo que tiene anotado tu obra, e Instrucciones, con este mismo texto. Solo hace falta escribir en las columnas de fondo amarillo, que son «Respuesta», «Excepciones / detalle» y «Comentario». El resto de columnas las genera el programa y las necesita tal cual para poder leer las respuestas, así que conviene no tocarlas.</t>
-  </si>
-  <si>
-    <t>En Responder están las preguntas que no hemos podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta. Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» explica el formato. Las preguntas que se refieren a cada estrofa aparecen de dos maneras: si son pocas estrofas, hay una fila por estrofa; si son muchas, hay una sola fila cuya respuesta vale para todas, y las estrofas que se aparten de ella se anotan en «Excepciones / detalle» indicando los versos y la respuesta, por ejemplo «191–194: Cruzada · abab; 203–206: Cruzada · abab».</t>
-  </si>
-  <si>
-    <t>Las filas marcadas como Decidir señalan pasajes cuyo número de versos no encaja con la forma que tienen asignada. En ellas hay que elegir en el desplegable qué ocurre y explicarlo al lado. Si se trata de una laguna que no se contó, indica en qué verso está y cuántos versos faltan, porque los añadiremos a la numeración y todo lo que viene después se desplazará. Si lo que falla es el rango, escribe el rango correcto.</t>
-  </si>
-  <si>
-    <t>En Confirmar aparecen las respuestas que hemos rellenado nosotros a partir del término que elegiste en su día: la asonancia de un romance, el esquema de una octava real «regular», o que un endecasílabo suelto «puro» no lleva pareados. Solo hay que revisarlas. Si alguna no es así, elige «No es así» y escribe al lado lo que corresponde.</t>
+    <t>Para María Isabel Cuena · generado el 2026-09-20</t>
+  </si>
+  <si>
+    <t>El Excel tiene cinco pestañas. En tres de ellas hay que escribir —Responder, Confirmar y Desviaciones— y las otras dos son de consulta: Secuencias, con todo lo que tiene anotado tu obra, e Instrucciones, donde estás ahora. Solo hace falta escribir en las columnas de fondo amarillo, que son «Respuesta», «Excepciones / detalle» y «Comentario». El resto de columnas las genera el programa y las necesita tal cual para poder leer las respuestas, así que conviene no tocarlas.</t>
+  </si>
+  <si>
+    <t>En Responder están las preguntas que no he podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta. Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» explica el formato. Las preguntas que se refieren a cada estrofa aparecen de dos maneras: si son pocas estrofas, hay una fila por estrofa; si son muchas, hay una sola fila cuya respuesta vale para todas, y las estrofas que se aparten de ella se anotan en «Excepciones / detalle» indicando los versos y la respuesta, por ejemplo «191–194: Cruzada · abab; 203–206: Cruzada · abab».</t>
+  </si>
+  <si>
+    <t>Las filas marcadas como Decidir señalan pasajes cuyo número de versos no encaja con la forma que tienen asignada. En ellas hay que elegir en el desplegable qué ocurre y explicarlo al lado. Si se trata de una laguna que no se contó, indica en qué verso está y cuántos versos faltan, porque los añadiré a la numeración y todo lo que viene después se desplazará. Si lo que falla es el rango, escribe el rango correcto.</t>
+  </si>
+  <si>
+    <t>En Confirmar aparecen las respuestas que he rellenado yo a partir del término que elegiste en su día: la asonancia de un romance, el esquema de una octava real «regular», o que un endecasílabo suelto «puro» no lleva pareados. Solo hay que revisarlas. Si alguna no es así, elige «No es así» y escribe al lado lo que corresponde.</t>
   </si>
   <si>
     <t>En Desviaciones están los versos hipométricos e hipermétricos, las rimas defectuosas y las lagunas que anotaste, con tus notas, y cómo quedan en el modelo nuevo. Se trasladan tal cual. Si tienes a mano el número de sílabas de algún verso hipométrico o hipermétrico, ponlo en la columna «Sílabas»; si no, se registra simplemente que el verso tiene menos o más sílabas de las que le tocan, sin dar una cifra.</t>
   </si>
   <si>
-    <t>Si algo no está claro o no sabes cómo contestarlo, pregúntaselo a David antes de dejarlo a medias. Una vez hecha la migración podrás ver cada secuencia de tu obra con el editor nuevo en el dashboard y corregir allí lo que haga falta.</t>
+    <t>Si algo no está claro o no sabes cómo contestarlo, pregúntamelo antes de dejarlo a medias. Una vez hecha la migración podrás ver cada secuencia de tu obra con el editor nuevo en el dashboard y comprobar allí que la migración no dejó ningún hueco.</t>
   </si>
   <si>
     <t>Cuando no hay desplegable, los formatos son estos:</t>
@@ -207,7 +207,7 @@
     <t>Redondilla · Octosílaba</t>
   </si>
   <si>
-    <t>Sus 225 versos no encajan con «Octosílaba», que se compone de unidades completas de 4 versos. Encajaría con 3 versos más (228) o con 1 verso menos (224).</t>
+    <t>Sus 225 versos no encajan en una redondilla octosílaba, que se compone de unidades completas de 4 versos. Encajaría con 3 versos más (228) o con 1 verso menos (224).</t>
   </si>
   <si>
     <t/>
@@ -225,7 +225,7 @@
     <t>Romance · Octosílabo</t>
   </si>
   <si>
-    <t>Tiene 53 versos, y un romance no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraremos la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
+    <t>Tiene 53 versos, y un romance octosílabo no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraré la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
   </si>
   <si>
     <t>L|6cc5851f-0ef9-41b7-8111-7b49f70b6bae</t>
@@ -234,7 +234,7 @@
     <t>787–885</t>
   </si>
   <si>
-    <t>Tiene 99 versos, y un romance no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraremos la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
+    <t>Tiene 99 versos, y un romance octosílabo no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraré la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
   </si>
   <si>
     <t>L|9655e7f1-89de-4565-9c55-54d9faf77031</t>
@@ -246,7 +246,7 @@
     <t>Seguidilla · Simple</t>
   </si>
   <si>
-    <t>Solo tiene 2 versos, y «Simple» necesita al menos 4. Puede que el rango esté mal o que se trate de otra forma.</t>
+    <t>Solo tiene 2 versos, y una seguidilla simple necesita al menos 4. Puede que el rango esté mal o que se trate de otra forma.</t>
   </si>
   <si>
     <t>L|83d7757a-99ef-4653-9fe2-1bcd1cb649af</t>
@@ -1389,10 +1389,10 @@
 hipometrico (276–276)</t>
   </si>
   <si>
-    <t>Revisar: Sus 225 versos no encajan con «Octosílaba», que se compone de unidades completas de 4 versos. Encajaría con 3 versos más (228) o con 1 verso menos (224).</t>
-  </si>
-  <si>
-    <t>Revisar: Tiene 53 versos, y un romance no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraremos la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
+    <t>Revisar: Sus 225 versos no encajan en una redondilla octosílaba, que se compone de unidades completas de 4 versos. Encajaría con 3 versos más (228) o con 1 verso menos (224).</t>
+  </si>
+  <si>
+    <t>Revisar: Tiene 53 versos, y un romance octosílabo no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraré la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
   </si>
   <si>
     <t>461–490</t>
@@ -1427,7 +1427,7 @@
 hipermetrico (878–878)</t>
   </si>
   <si>
-    <t>Revisar: Tiene 99 versos, y un romance no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraremos la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
+    <t>Revisar: Tiene 99 versos, y un romance octosílabo no puede tener un número impar: en algún punto falta o sobra un verso. Hay que localizarlo y decir si se trata de una laguna, en cuyo caso renumeraré la obra a partir de ahí, o de un error en el rango, en cuyo caso hace falta el rango correcto.</t>
   </si>
   <si>
     <t>seguidilla</t>
@@ -1439,7 +1439,7 @@
     <t>Simple</t>
   </si>
   <si>
-    <t>Revisar: Solo tiene 2 versos, y «Simple» necesita al menos 4. Puede que el rango esté mal o que se trate de otra forma.</t>
+    <t>Revisar: Solo tiene 2 versos, y una seguidilla simple necesita al menos 4. Puede que el rango esté mal o que se trate de otra forma.</t>
   </si>
   <si>
     <t xml:space="preserve">hipometrico (961–961)

</xml_diff>